<commit_message>
hw: set U1, J1, C1 to DNP in assembly BOM for resistor-only assembly
</commit_message>
<xml_diff>
--- a/hardware/C5VRX_JACK_DIY/BOM-assembly.xlsx
+++ b/hardware/C5VRX_JACK_DIY/BOM-assembly.xlsx
@@ -668,7 +668,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>470pF 50V C0G ceramic disc capacitor (P2.5mm); DNP (optional RF filter)</t>
+          <t>DO NOT POPULATE (leave unpopulated)</t>
         </is>
       </c>
     </row>
@@ -691,12 +691,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>DNP</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>9-pin 1x09 right-angle 2.54mm male header for Fat Shark goggle bay</t>
+          <t>DO NOT POPULATE (leave unpopulated)</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>DNP</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>4-pole TRRS SMD 3.5mm phone jack facing left (PJ-320D)</t>
+          <t>DO NOT POPULATE (leave unpopulated)</t>
         </is>
       </c>
     </row>
@@ -738,21 +738,21 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PPTC071LFBN-RC</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>DNP</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2x 1x07 2.54mm female header sockets for Seeed XIAO ESP32-C5 (XIAO module plugged in by customer)</t>
+          <t>DO NOT POPULATE (leave unpopulated; user solders XIAO)</t>
         </is>
       </c>
     </row>

</xml_diff>